<commit_message>
Se continua con el proceso de limpieza de datos.
</commit_message>
<xml_diff>
--- a/limpieza_dataset_alumnos/DatosExamen.xlsx
+++ b/limpieza_dataset_alumnos/DatosExamen.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Documents\Ingeniería de Datos\repositorio\Ingenierina_de_datos\limpieza_dataset_alumnos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EFA86A3-37E1-45F6-B383-C80D9CCBA555}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5601E3C-CB7A-4B90-A5DE-5D983BD3847C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="147">
   <si>
     <t>Nombre</t>
   </si>
@@ -437,28 +437,49 @@
     <t>('Carlos Enrique Figueroa Solano', '21', 'Xalapa, Veracruz', '9', '11/10/2003', 'Coyoacán', 'Si', 'Bimbo', '9no', 'Es la ciencia de resolver problemas', 'Es la parte más pequeña de la información', 'Nothing But Thieves', 'Fotografía, videojuegos, escuchar música', '2', 'Cálculo Vectorial, Estructura de datos y algoritmos, dispositivos'),</t>
   </si>
   <si>
-    <t>('Gómez Urbano Mariana', '22 años', 'Edo. Méx, Chimalhuacán', '45908', '06/nov/2022', 'Chimalhuacán', 'No', '', '10', 'Disciplina que engloba múltiples conocimientos técnicos y científicos con el fin de diseñar e implementar soluciones innovadoras', 'Es una representación de sucesos, carácteristicas; por lo regular un dato no tiene significado por si solo necesita ser tratado para llegar a ser información', 'Miku', 'Ver series, leer manwas, salir a caminar', 'En copilco somos 2, en mi casa 5', ''),</t>
-  </si>
-  <si>
-    <t>('Jonathan Reyes Ramírez', '25 años', 'Estado de México', '45877', '26 de marzo del 2000', 'Ocoyoacac, Estado de México', 'No', '', '11vo semestre', 'Es el "arte" o forma en que conocimiento teorico se lleva a la practica, ya sea para solucionar un problema, innovar o crear tecnología', 'Es información que puede estar guardada en diferentes formatos y que nos sirve para entender algo', 'Royal Blod', 'Ver películas, Escuchar musica, caminar/correr por la naturaleza', '3', 'Calculo y Geometría analítica, Sistemas de comunicaciones. Sistemas operativos'),</t>
-  </si>
-  <si>
     <t>('Carlos Ceniceros Moriaca', '23', 'Ciudad de México', '8.56', '24 de agosto de 2001', 'Tizayuca Hidalgo', 'No trabajo', '', 'Estoy en mi onceavo semestre', 'La disciplina encargada de aplicar la teoría en beneficio de un fin', 'La unidad minima de la información', 'Sabatan', 'Descansar, ver peliculas, jugar videojuegos', '3', 'Bases de datos, Redes de Datos seguras, EDA2'),</t>
   </si>
   <si>
-    <t>('Ernesto Quintana López', '22 años', 'Tuxtepec, Oaxaca', '45666', '6/Diciembre/2002', 'Coyoacan', 'No', '', '9', 'El conocimiento que se utiliza para realizar cosas con ingenio', 'Representación de un pequeño fragmento de información', 'Cuarteto de Nos', 'Correr,Escuchar musica y cocinar', 'Nadie', 'POO,Calculo y Geometria Analitica y BD'),</t>
-  </si>
-  <si>
     <t>('Laylet Rojas Terrazas', '26 años ', 'México D.F -&gt; CDMX', '9.65', '19 de octubre de 1998', 'Benito Juárez ', 'Si', 'Trabajo en PepsiCo en CMDB, "Data Governance"', 'Onceavo semestre', 'Conjunto de Ciencias aplicadas para diseñar, construir soluciones óptimas y facilitar la vida ', 'Mínima información, por si solo no tiene significado', 'Coldplay ', 'Tocar piano, hacer ejercicio (artes mixtas), cocinar ', '3 personas más ', 'Bases de datos (todas), Cisco, cálculo y geometriía analítica, lenguajes autómatas '),</t>
+  </si>
+  <si>
+    <t>8.78</t>
+  </si>
+  <si>
+    <t>8.5</t>
+  </si>
+  <si>
+    <t>9.21</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>8.9</t>
+  </si>
+  <si>
+    <t>8.8</t>
+  </si>
+  <si>
+    <t>8.56</t>
+  </si>
+  <si>
+    <t>9.1</t>
+  </si>
+  <si>
+    <t>('Gómez Urbano Mariana', '22 años', 'Edo. Méx, Chimalhuacán', '8.9', '06/nov/2022', 'Chimalhuacán', 'No', '', '10', 'Disciplina que engloba múltiples conocimientos técnicos y científicos con el fin de diseñar e implementar soluciones innovadoras', 'Es una representación de sucesos, carácteristicas; por lo regular un dato no tiene significado por si solo necesita ser tratado para llegar a ser información', 'Miku', 'Ver series, leer manwas, salir a caminar', 'En copilco somos 2, en mi casa 5', ''),</t>
+  </si>
+  <si>
+    <t>('Jonathan Reyes Ramírez', '25 años', 'Estado de México', '8.8', '26 de marzo del 2000', 'Ocoyoacac, Estado de México', 'No', '', '11vo semestre', 'Es el "arte" o forma en que conocimiento teorico se lleva a la practica, ya sea para solucionar un problema, innovar o crear tecnología', 'Es información que puede estar guardada en diferentes formatos y que nos sirve para entender algo', 'Royal Blod', 'Ver películas, Escuchar musica, caminar/correr por la naturaleza', '3', 'Calculo y Geometría analítica, Sistemas de comunicaciones. Sistemas operativos'),</t>
+  </si>
+  <si>
+    <t>('Ernesto Quintana López', '22 años', 'Tuxtepec, Oaxaca', '9.1', '6/Diciembre/2002', 'Coyoacan', 'No', '', '9', 'El conocimiento que se utiliza para realizar cosas con ingenio', 'Representación de un pequeño fragmento de información', 'Cuarteto de Nos', 'Correr,Escuchar musica y cocinar', 'Nadie', 'POO,Calculo y Geometria Analitica y BD'),</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="d\.m"/>
-  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -479,12 +500,24 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF6F8F9"/>
+        <bgColor rgb="FFF6F8F9"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="13">
@@ -679,7 +712,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -721,12 +754,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -741,6 +768,19 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -759,6 +799,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
+      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
       <font>
@@ -1025,23 +1066,23 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla_1" displayName="Tabla_1" ref="A1:O11" headerRowDxfId="2" dataDxfId="0" totalsRowDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla_1" displayName="Tabla_1" ref="A1:O11" headerRowDxfId="17" dataDxfId="16" totalsRowDxfId="15">
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Nombre" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Edad" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Lugar de Nacimiento" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Promedio" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Fecha de Nacimiento" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Donde Vivo" dataDxfId="12"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Trabajo" dataDxfId="11"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Dónde Trabajo" dataDxfId="10"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Semestre" dataDxfId="9"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Ingeniería" dataDxfId="8"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Dato" dataDxfId="7"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Artista Favorito" dataDxfId="6"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="3 hobbies" dataDxfId="5"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Con cuantos vivo" dataDxfId="4"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="3 Materias Favoritas" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Nombre" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Edad" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Lugar de Nacimiento" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Promedio" dataDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Fecha de Nacimiento" dataDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Donde Vivo" dataDxfId="10"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Trabajo" dataDxfId="9"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Dónde Trabajo" dataDxfId="8"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Semestre" dataDxfId="7"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Ingeniería" dataDxfId="6"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Dato" dataDxfId="5"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Artista Favorito" dataDxfId="4"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="3 hobbies" dataDxfId="3"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Con cuantos vivo" dataDxfId="2"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="3 Materias Favoritas" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="Hoja 1-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1254,7 +1295,7 @@
     <col min="1" max="1" width="30" style="4" customWidth="1"/>
     <col min="2" max="2" width="12.59765625" style="4"/>
     <col min="3" max="3" width="25.3984375" style="4" customWidth="1"/>
-    <col min="4" max="4" width="19.3984375" style="4" customWidth="1"/>
+    <col min="4" max="4" width="19.3984375" style="21" customWidth="1"/>
     <col min="5" max="5" width="24.3984375" style="4" customWidth="1"/>
     <col min="6" max="6" width="26.5" style="4" customWidth="1"/>
     <col min="7" max="7" width="12.59765625" style="4"/>
@@ -1266,10 +1307,12 @@
     <col min="13" max="13" width="51.19921875" style="4" customWidth="1"/>
     <col min="14" max="14" width="32" style="4" customWidth="1"/>
     <col min="15" max="15" width="67.8984375" style="4" customWidth="1"/>
-    <col min="16" max="16384" width="12.59765625" style="4"/>
+    <col min="16" max="16" width="12.59765625" style="4"/>
+    <col min="17" max="17" width="58.296875" style="4" customWidth="1"/>
+    <col min="18" max="16384" width="12.59765625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1279,7 +1322,7 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="20" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
@@ -1316,7 +1359,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>15</v>
       </c>
@@ -1326,8 +1369,8 @@
       <c r="C2" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="6">
-        <v>8.7799999999999994</v>
+      <c r="D2" s="22" t="s">
+        <v>136</v>
       </c>
       <c r="E2" s="7" t="s">
         <v>17</v>
@@ -1368,7 +1411,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>26</v>
       </c>
@@ -1378,8 +1421,8 @@
       <c r="C3" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="D3" s="11">
-        <v>8.5</v>
+      <c r="D3" s="23" t="s">
+        <v>137</v>
       </c>
       <c r="E3" s="12" t="s">
         <v>28</v>
@@ -1418,7 +1461,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>35</v>
       </c>
@@ -1428,8 +1471,8 @@
       <c r="C4" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="D4" s="6">
-        <v>9.2100000000000009</v>
+      <c r="D4" s="22" t="s">
+        <v>138</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>37</v>
@@ -1472,7 +1515,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>48</v>
       </c>
@@ -1482,7 +1525,7 @@
       <c r="C5" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="23" t="s">
         <v>51</v>
       </c>
       <c r="E5" s="12" t="s">
@@ -1526,7 +1569,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>62</v>
       </c>
@@ -1536,8 +1579,8 @@
       <c r="C6" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="D6" s="6">
-        <v>9</v>
+      <c r="D6" s="22" t="s">
+        <v>139</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>64</v>
@@ -1580,7 +1623,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>73</v>
       </c>
@@ -1590,8 +1633,8 @@
       <c r="C7" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="D7" s="15">
-        <v>45908</v>
+      <c r="D7" s="23" t="s">
+        <v>140</v>
       </c>
       <c r="E7" s="12" t="s">
         <v>76</v>
@@ -1624,13 +1667,13 @@
       <c r="O7" s="14"/>
       <c r="Q7" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>('Gómez Urbano Mariana', '22 años', 'Edo. Méx, Chimalhuacán', '45908', '06/nov/2022', 'Chimalhuacán', 'No', '', '10', 'Disciplina que engloba múltiples conocimientos técnicos y científicos con el fin de diseñar e implementar soluciones innovadoras', 'Es una representación de sucesos, carácteristicas; por lo regular un dato no tiene significado por si solo necesita ser tratado para llegar a ser información', 'Miku', 'Ver series, leer manwas, salir a caminar', 'En copilco somos 2, en mi casa 5', ''),</v>
+        <v>('Gómez Urbano Mariana', '22 años', 'Edo. Méx, Chimalhuacán', '8.9', '06/nov/2022', 'Chimalhuacán', 'No', '', '10', 'Disciplina que engloba múltiples conocimientos técnicos y científicos con el fin de diseñar e implementar soluciones innovadoras', 'Es una representación de sucesos, carácteristicas; por lo regular un dato no tiene significado por si solo necesita ser tratado para llegar a ser información', 'Miku', 'Ver series, leer manwas, salir a caminar', 'En copilco somos 2, en mi casa 5', ''),</v>
       </c>
       <c r="R7" s="4" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>83</v>
       </c>
@@ -1640,8 +1683,8 @@
       <c r="C8" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="D8" s="16">
-        <v>45877</v>
+      <c r="D8" s="22" t="s">
+        <v>141</v>
       </c>
       <c r="E8" s="7" t="s">
         <v>86</v>
@@ -1676,13 +1719,13 @@
       </c>
       <c r="Q8" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>('Jonathan Reyes Ramírez', '25 años', 'Estado de México', '45877', '26 de marzo del 2000', 'Ocoyoacac, Estado de México', 'No', '', '11vo semestre', 'Es el "arte" o forma en que conocimiento teorico se lleva a la practica, ya sea para solucionar un problema, innovar o crear tecnología', 'Es información que puede estar guardada en diferentes formatos y que nos sirve para entender algo', 'Royal Blod', 'Ver películas, Escuchar musica, caminar/correr por la naturaleza', '3', 'Calculo y Geometría analítica, Sistemas de comunicaciones. Sistemas operativos'),</v>
+        <v>('Jonathan Reyes Ramírez', '25 años', 'Estado de México', '8.8', '26 de marzo del 2000', 'Ocoyoacac, Estado de México', 'No', '', '11vo semestre', 'Es el "arte" o forma en que conocimiento teorico se lleva a la practica, ya sea para solucionar un problema, innovar o crear tecnología', 'Es información que puede estar guardada en diferentes formatos y que nos sirve para entender algo', 'Royal Blod', 'Ver películas, Escuchar musica, caminar/correr por la naturaleza', '3', 'Calculo y Geometría analítica, Sistemas de comunicaciones. Sistemas operativos'),</v>
       </c>
       <c r="R8" s="4" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>94</v>
       </c>
@@ -1692,8 +1735,8 @@
       <c r="C9" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="D9" s="11">
-        <v>8.56</v>
+      <c r="D9" s="23" t="s">
+        <v>142</v>
       </c>
       <c r="E9" s="12" t="s">
         <v>96</v>
@@ -1731,10 +1774,10 @@
         <v>('Carlos Ceniceros Moriaca', '23', 'Ciudad de México', '8.56', '24 de agosto de 2001', 'Tizayuca Hidalgo', 'No trabajo', '', 'Estoy en mi onceavo semestre', 'La disciplina encargada de aplicar la teoría en beneficio de un fin', 'La unidad minima de la información', 'Sabatan', 'Descansar, ver peliculas, jugar videojuegos', '3', 'Bases de datos, Redes de Datos seguras, EDA2'),</v>
       </c>
       <c r="R9" s="4" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>105</v>
       </c>
@@ -1744,8 +1787,8 @@
       <c r="C10" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="D10" s="16">
-        <v>45666</v>
+      <c r="D10" s="22" t="s">
+        <v>143</v>
       </c>
       <c r="E10" s="7" t="s">
         <v>107</v>
@@ -1780,56 +1823,56 @@
       </c>
       <c r="Q10" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>('Ernesto Quintana López', '22 años', 'Tuxtepec, Oaxaca', '45666', '6/Diciembre/2002', 'Coyoacan', 'No', '', '9', 'El conocimiento que se utiliza para realizar cosas con ingenio', 'Representación de un pequeño fragmento de información', 'Cuarteto de Nos', 'Correr,Escuchar musica y cocinar', 'Nadie', 'POO,Calculo y Geometria Analitica y BD'),</v>
+        <v>('Ernesto Quintana López', '22 años', 'Tuxtepec, Oaxaca', '9.1', '6/Diciembre/2002', 'Coyoacan', 'No', '', '9', 'El conocimiento que se utiliza para realizar cosas con ingenio', 'Representación de un pequeño fragmento de información', 'Cuarteto de Nos', 'Correr,Escuchar musica y cocinar', 'Nadie', 'POO,Calculo y Geometria Analitica y BD'),</v>
       </c>
       <c r="R10" s="4" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A11" s="17" t="s">
+    <row r="11" spans="1:18" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A11" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="16" t="s">
         <v>115</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="16" t="s">
         <v>116</v>
       </c>
-      <c r="D11" s="18" t="s">
+      <c r="D11" s="24" t="s">
         <v>117</v>
       </c>
-      <c r="E11" s="19" t="s">
+      <c r="E11" s="17" t="s">
         <v>118</v>
       </c>
-      <c r="F11" s="18" t="s">
+      <c r="F11" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="G11" s="18" t="s">
+      <c r="G11" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="H11" s="18" t="s">
+      <c r="H11" s="16" t="s">
         <v>120</v>
       </c>
-      <c r="I11" s="18" t="s">
+      <c r="I11" s="16" t="s">
         <v>121</v>
       </c>
-      <c r="J11" s="18" t="s">
+      <c r="J11" s="16" t="s">
         <v>122</v>
       </c>
-      <c r="K11" s="18" t="s">
+      <c r="K11" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="L11" s="18" t="s">
+      <c r="L11" s="16" t="s">
         <v>124</v>
       </c>
-      <c r="M11" s="20" t="s">
+      <c r="M11" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="N11" s="18" t="s">
+      <c r="N11" s="16" t="s">
         <v>126</v>
       </c>
-      <c r="O11" s="21" t="s">
+      <c r="O11" s="19" t="s">
         <v>127</v>
       </c>
       <c r="Q11" s="4" t="str">
@@ -1837,7 +1880,7 @@
         <v>('Laylet Rojas Terrazas', '26 años ', 'México D.F -&gt; CDMX', '9.65', '19 de octubre de 1998', 'Benito Juárez ', 'Si', 'Trabajo en PepsiCo en CMDB, "Data Governance"', 'Onceavo semestre', 'Conjunto de Ciencias aplicadas para diseñar, construir soluciones óptimas y facilitar la vida ', 'Mínima información, por si solo no tiene significado', 'Coldplay ', 'Tocar piano, hacer ejercicio (artes mixtas), cocinar ', '3 personas más ', 'Bases de datos (todas), Cisco, cálculo y geometriía analítica, lenguajes autómatas '),</v>
       </c>
       <c r="R11" s="4" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="12" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>